<commit_message>
Number worksheet URL directories as 001 and 002
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ymdjz" sheetId="1" r:id="R0d479c53517f482f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2消失的龙" sheetId="3" r:id="R3688fc072da748ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="001" sheetId="1" r:id="R0d479c53517f482f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="002" sheetId="3" r:id="R3688fc072da748ee"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
add tips and  an image
add tips and  an image
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15360"/>
+    <workbookView windowHeight="23960"/>
   </bookViews>
   <sheets>
     <sheet name="001" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>网址</t>
   </si>
@@ -42,41 +42,41 @@
     <t>ch1-1</t>
   </si>
   <si>
-    <t>日记中的古诗提到两处古迹的名字，有一处现已无存，请找到仍然存在的古迹名称，即为答案。</t>
+    <t>日记中提到一处有点玄的古迹的名字，即为答案。</t>
   </si>
   <si>
     <t>ch1-2-1</t>
   </si>
   <si>
-    <t>请找到《皇都篇》碑文拓片。碑文末尾的落款纪年，与现场石碑基座束腰处的水兽数目，共同组成4位数字密码。</t>
+    <t>请找到找到那张绘有石刻装饰局部的硫酸纸，把他与日记背面的碑文相叠，与石刻装饰位置对应的碑文，就是密语。密语中有一个不常见的字。“衢”，读作 qú，指四通八达的道路。</t>
   </si>
   <si>
     <t>ch1-2-2</t>
   </si>
   <si>
-    <t>《皇都篇》碑文末尾的落款纪年，即为密码前两位；石碑基座束腰处水兽的数量，即为后两位。</t>
+    <t>密语中十个字的顺序，来自于石刻装饰在燕墩石碑上“从上到下、从左到右”的顺序。</t>
   </si>
   <si>
     <t>ch1-2-3</t>
   </si>
   <si>
-    <t xml:space="preserve">水兽并不在碑身，而在石碑基座束腰处，基座有四面，不要遗漏任何一面。
+    <t xml:space="preserve">
 </t>
   </si>
   <si>
+    <t>images/ch1-2-3.png</t>
+  </si>
+  <si>
     <t>ch1-3-1</t>
   </si>
   <si>
-    <t>《日下旧闻考》中，有一句话被用蓝线标记出来。这句话描述了燕墩和下一处地点的位置关系。 -</t>
+    <t>除了“城楼北偏东”的指引之外，你还可以回头去看之前贴在日记上的《日下旧闻考》，那句被用蓝线划出来的话描述了燕墩和下一处地点的位置关系和距离。</t>
   </si>
   <si>
     <t>ch1-3-2</t>
   </si>
   <si>
-    <t>请将那幅城门楼的彩画与现场的城门楼进行比对。找到不同之后，你会发现这处不同所对应的数字坐标。 - -如遇城楼修缮，现场无法完成调查，请退出当前页面，点击「求助提示3」。</t>
+    <t>请将那幅城门楼的彩画与现场的城门楼进行比对。找到不同之后，你会发现这处不同所对应的数字坐标。</t>
   </si>
   <si>
     <t>ch1-3-3</t>
@@ -127,8 +127,7 @@
     <t>ch1-7-1</t>
   </si>
   <si>
-    <t xml:space="preserve">请对照《天桥盛景图》，在现实中找到画中的天桥。石碑，就在它旁边。
-</t>
+    <t>请对照《天桥盛景图》，在现实中找到画中的那座石拱桥，也就是北京中轴线上的祭天之桥——“天桥”。而石碑，就在它旁边</t>
   </si>
   <si>
     <t>ch1-7-2</t>
@@ -143,15 +142,30 @@
     <t>ch1-8-1</t>
   </si>
   <si>
-    <t>请开启调查资料中封存的*最终附件*中的《碑刻龙纹初考》，你会发现有六条龙纹改变了视线。</t>
+    <t>请务必站在石碑的南面观察</t>
   </si>
   <si>
     <t>ch1-8-2</t>
   </si>
   <si>
-    <t xml:space="preserve">在碑文的四周共有14条龙，其中有三组龙，每组两条，彼此相望。
+    <t>在右上角、右下角，左上角，左下角中回答一个</t>
+  </si>
+  <si>
+    <t>ch1-9-1</t>
+  </si>
+  <si>
+    <t>在《碑刻龙纹初考》的背面有一首诗，留意诗中信息</t>
+  </si>
+  <si>
+    <t>ch1-9-2</t>
+  </si>
+  <si>
+    <t>“连”紋对照目相“接”，“龙”影相望各回“头” +“一”痕暗刻舊石中，“三”分無言訴春秋 +“四”顧城南尋往事，遍覓“十有一”處幽 +“八”方尋跡龍紋隱，“双七”相見意未休
  -请用直线分别连接每对互相对望的两条龙的龙眼，当三对目光彼此相遇时，答案便会显现。 </t>
+连接龙头，1和3，4和11，8和14</t>
   </si>
 </sst>
 </file>
@@ -1253,7 +1267,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="17.6" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1272,7 +1286,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="28.8" customHeight="1" spans="1:3">
+    <row r="2" ht="54" customHeight="1" spans="1:3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1280,7 +1294,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" ht="43.2" customHeight="1" spans="1:3">
+    <row r="3" ht="86" customHeight="1" spans="1:3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1288,7 +1302,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="28.8" customHeight="1" spans="1:3">
+    <row r="4" ht="51" customHeight="1" spans="1:3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1303,114 +1317,130 @@
       <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" ht="28.8" customHeight="1" spans="1:3">
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" ht="69" customHeight="1" spans="1:3">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" ht="57.6" customHeight="1" spans="1:3">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:3">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" ht="28.8" customHeight="1" spans="1:3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" spans="1:3">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" ht="43.2" customHeight="1" spans="1:3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" ht="71" customHeight="1" spans="1:3">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" ht="28.8" customHeight="1" spans="1:3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" ht="53" customHeight="1" spans="1:3">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" ht="28.8" customHeight="1" spans="1:3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1" spans="1:3">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:3">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" ht="57.6" customHeight="1" spans="1:3">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="15" ht="45.6" customHeight="1" spans="1:3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" ht="69" customHeight="1" spans="1:3">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" ht="88.8" customHeight="1" spans="1:3">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" ht="28.8" customHeight="1" spans="1:2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" ht="78" customHeight="1" spans="1:2">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" ht="57.6" customHeight="1" spans="1:2">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="B19"/>
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" ht="71" spans="1:2">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>